<commit_message>
updated output sheets and created recordings from paraview to show other people
</commit_message>
<xml_diff>
--- a/examples/Methylene Blue Diffusion Parameter Fitting/drug-eluting hydrogel implants.jl/drug_eluting_hydrogel_implant_fever_natural_diffusion_results.xlsx
+++ b/examples/Methylene Blue Diffusion Parameter Fitting/drug-eluting hydrogel implants.jl/drug_eluting_hydrogel_implant_fever_natural_diffusion_results.xlsx
@@ -403,1602 +403,1602 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>3024.0</v>
+        <v>18.0</v>
       </c>
       <c r="B3">
-        <v>3.5521260710758556e-57</v>
+        <v>1.5908462680831379e-25</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>6048.0</v>
+        <v>36.0</v>
       </c>
       <c r="B4">
-        <v>1.1549670336771409e-52</v>
+        <v>4.6444512473189983e-20</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>9072.0</v>
+        <v>54.0</v>
       </c>
       <c r="B5">
-        <v>8.92161555648029e-49</v>
+        <v>2.899675427744029e-17</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>12096.0</v>
+        <v>72.0</v>
       </c>
       <c r="B6">
-        <v>3.1138309793623736e-48</v>
+        <v>1.57878417381121e-15</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>15120.0</v>
+        <v>90.0</v>
       </c>
       <c r="B7">
-        <v>6.542231349252595e-48</v>
+        <v>3.3008119716598173e-14</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>18144.0</v>
+        <v>108.0</v>
       </c>
       <c r="B8">
-        <v>5.790025624238836e-44</v>
+        <v>3.0515834810748623e-13</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>21168.0</v>
+        <v>126.0</v>
       </c>
       <c r="B9">
-        <v>1.4788874395245998e-43</v>
+        <v>1.7642618034949177e-12</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>24192.0</v>
+        <v>144.0</v>
       </c>
       <c r="B10">
-        <v>2.691430790681083e-43</v>
+        <v>8.228966608058363e-12</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>27216.0</v>
+        <v>162.0</v>
       </c>
       <c r="B11">
-        <v>4.2166326158933354e-43</v>
+        <v>3.2339111355627336e-11</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>30240.0</v>
+        <v>180.0</v>
       </c>
       <c r="B12">
-        <v>6.054492915161356e-43</v>
+        <v>9.86188805624141e-11</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>33264.0</v>
+        <v>198.0</v>
       </c>
       <c r="B13">
-        <v>8.205011688485146e-43</v>
+        <v>2.8033475906686914e-10</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>36288.0</v>
+        <v>216.0</v>
       </c>
       <c r="B14">
-        <v>1.06681889358647e-42</v>
+        <v>6.844814347297366e-10</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>39312.0</v>
+        <v>234.0</v>
       </c>
       <c r="B15">
-        <v>3.459066829200946e-39</v>
+        <v>1.58107039251084e-9</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>42336.0</v>
+        <v>252.0</v>
       </c>
       <c r="B16">
-        <v>8.353995263799565e-38</v>
+        <v>3.209710133161962e-9</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>45360.0</v>
+        <v>270.0</v>
       </c>
       <c r="B17">
-        <v>1.8135793062182764e-37</v>
+        <v>6.28584397469062e-9</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>48384.0</v>
+        <v>288.0</v>
       </c>
       <c r="B18">
-        <v>2.9691300078069687e-37</v>
+        <v>1.1345201681396862e-8</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>51408.0</v>
+        <v>306.0</v>
       </c>
       <c r="B19">
-        <v>4.302051631146033e-37</v>
+        <v>1.940947451548581e-8</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>54432.0</v>
+        <v>324.0</v>
       </c>
       <c r="B20">
-        <v>5.812344176235471e-37</v>
+        <v>3.2046601739322515e-8</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>57456.0</v>
+        <v>342.0</v>
       </c>
       <c r="B21">
-        <v>7.500007643075283e-37</v>
+        <v>5.0820456405630004e-8</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>60480.0</v>
+        <v>360.0</v>
       </c>
       <c r="B22">
-        <v>9.365042031665464e-37</v>
+        <v>7.887925691001522e-8</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>63504.0</v>
+        <v>378.0</v>
       </c>
       <c r="B23">
-        <v>1.1407447342006023e-36</v>
+        <v>1.178355872757321e-7</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>66528.0</v>
+        <v>396.0</v>
       </c>
       <c r="B24">
-        <v>1.362722357409695e-36</v>
+        <v>1.693599010077723e-7</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>69552.0</v>
+        <v>414.0</v>
       </c>
       <c r="B25">
-        <v>1.6024370727938247e-36</v>
+        <v>2.384582085786091e-7</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>72576.0</v>
+        <v>432.0</v>
       </c>
       <c r="B26">
-        <v>1.8598888803529926e-36</v>
+        <v>3.268141361604106e-7</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>75600.0</v>
+        <v>450.0</v>
       </c>
       <c r="B27">
-        <v>2.1350777800871975e-36</v>
+        <v>4.3700886856245554e-7</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>78624.0</v>
+        <v>468.0</v>
       </c>
       <c r="B28">
-        <v>2.428003771996439e-36</v>
+        <v>5.742848300457287e-7</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
-        <v>81648.0</v>
+        <v>486.0</v>
       </c>
       <c r="B29">
-        <v>2.7386668560807184e-36</v>
+        <v>7.406868562223275e-7</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30">
-        <v>84672.0</v>
+        <v>504.0</v>
       </c>
       <c r="B30">
-        <v>3.067067032340035e-36</v>
+        <v>9.392932199932586e-7</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31">
-        <v>87696.0</v>
+        <v>522.0</v>
       </c>
       <c r="B31">
-        <v>3.413204300774389e-36</v>
+        <v>1.1742702828814054e-6</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32">
-        <v>90720.0</v>
+        <v>540.0</v>
       </c>
       <c r="B32">
-        <v>3.77707866138378e-36</v>
+        <v>1.4488989923340507e-6</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33">
-        <v>93744.0</v>
+        <v>558.0</v>
       </c>
       <c r="B33">
-        <v>4.1586901141682075e-36</v>
+        <v>1.7657494430063614e-6</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34">
-        <v>96768.0</v>
+        <v>576.0</v>
       </c>
       <c r="B34">
-        <v>4.558038659127674e-36</v>
+        <v>2.1265813063589826e-6</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35">
-        <v>99792.0</v>
+        <v>594.0</v>
       </c>
       <c r="B35">
-        <v>4.9751242962621756e-36</v>
+        <v>2.535079956370808e-6</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36">
-        <v>102816.0</v>
+        <v>612.0</v>
       </c>
       <c r="B36">
-        <v>5.409947025571717e-36</v>
+        <v>2.9949514102294136e-6</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37">
-        <v>105840.0</v>
+        <v>630.0</v>
       </c>
       <c r="B37">
-        <v>5.862506847056295e-36</v>
+        <v>3.506451879028787e-6</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38">
-        <v>108864.0</v>
+        <v>648.0</v>
       </c>
       <c r="B38">
-        <v>6.332803760715908e-36</v>
+        <v>4.070382567158373e-6</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39">
-        <v>111888.0</v>
+        <v>666.0</v>
       </c>
       <c r="B39">
-        <v>6.820837766550561e-36</v>
+        <v>4.689131122378325e-6</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40">
-        <v>114912.0</v>
+        <v>684.0</v>
       </c>
       <c r="B40">
-        <v>7.326608864560248e-36</v>
+        <v>5.365085192448793e-6</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41">
-        <v>117936.0</v>
+        <v>702.0</v>
       </c>
       <c r="B41">
-        <v>7.850117054744976e-36</v>
+        <v>6.09876200468757e-6</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42">
-        <v>120960.0</v>
+        <v>720.0</v>
       </c>
       <c r="B42">
-        <v>8.391362337104741e-36</v>
+        <v>6.887976949306081e-6</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43">
-        <v>123984.0</v>
+        <v>738.0</v>
       </c>
       <c r="B43">
-        <v>8.950344711639541e-36</v>
+        <v>7.733113698346889e-6</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44">
-        <v>127008.0</v>
+        <v>756.0</v>
       </c>
       <c r="B44">
-        <v>9.527064178349379e-36</v>
+        <v>8.634626162821657e-6</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45">
-        <v>130032.0</v>
+        <v>774.0</v>
       </c>
       <c r="B45">
-        <v>1.0121520737234255e-35</v>
+        <v>9.592968253742057e-6</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46">
-        <v>133056.0</v>
+        <v>792.0</v>
       </c>
       <c r="B46">
-        <v>9.536023698174898e-33</v>
+        <v>1.0608457393322957e-5</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47">
-        <v>136080.0</v>
+        <v>810.0</v>
       </c>
       <c r="B47">
-        <v>1.2482460900732669e-31</v>
+        <v>1.1678768353637805e-5</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48">
-        <v>139104.0</v>
+        <v>828.0</v>
       </c>
       <c r="B48">
-        <v>2.472885810532647e-31</v>
+        <v>1.2801630750937039e-5</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49">
-        <v>142128.0</v>
+        <v>846.0</v>
       </c>
       <c r="B49">
-        <v>3.769279398359892e-31</v>
+        <v>1.3975353784818569e-5</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50">
-        <v>145152.0</v>
+        <v>864.0</v>
       </c>
       <c r="B50">
-        <v>5.137426853554999e-31</v>
+        <v>1.519824665488032e-5</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51">
-        <v>148176.0</v>
+        <v>882.0</v>
       </c>
       <c r="B51">
-        <v>6.577328176117968e-31</v>
+        <v>1.64686185607202e-5</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52">
-        <v>151200.0</v>
+        <v>900.0</v>
       </c>
       <c r="B52">
-        <v>8.0889833660488e-31</v>
+        <v>1.778551428594742e-5</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53">
-        <v>154224.0</v>
+        <v>918.0</v>
       </c>
       <c r="B53">
-        <v>9.672392423347497e-31</v>
+        <v>1.914802764842586e-5</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54">
-        <v>157248.0</v>
+        <v>936.0</v>
       </c>
       <c r="B54">
-        <v>1.1327555348014052e-30</v>
+        <v>2.0552804717593653e-5</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55">
-        <v>160272.0</v>
+        <v>954.0</v>
       </c>
       <c r="B55">
-        <v>1.3054472140048473e-30</v>
+        <v>2.1996408398297965e-5</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56">
-        <v>163296.0</v>
+        <v>972.0</v>
       </c>
       <c r="B56">
-        <v>1.4853142799450757e-30</v>
+        <v>2.3475401595385955e-5</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57">
-        <v>166320.0</v>
+        <v>990.0</v>
       </c>
       <c r="B57">
-        <v>1.6723567326220905e-30</v>
+        <v>2.4986544504556035e-5</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58">
-        <v>169344.0</v>
+        <v>1008.0</v>
       </c>
       <c r="B58">
-        <v>1.8665745720358914e-30</v>
+        <v>2.6531218311130343e-5</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59">
-        <v>172368.0</v>
+        <v>1026.0</v>
       </c>
       <c r="B59">
-        <v>2.067967798186479e-30</v>
+        <v>2.810814674721107e-5</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60">
-        <v>175392.0</v>
+        <v>1044.0</v>
       </c>
       <c r="B60">
-        <v>2.2765364110738528e-30</v>
+        <v>2.971401889224117e-5</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61">
-        <v>178416.0</v>
+        <v>1062.0</v>
       </c>
       <c r="B61">
-        <v>2.492280410698012e-30</v>
+        <v>3.134552382566359e-5</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62">
-        <v>181440.0</v>
+        <v>1080.0</v>
       </c>
       <c r="B62">
-        <v>2.7151997970589574e-30</v>
+        <v>3.299935062692129e-5</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63">
-        <v>184464.0</v>
+        <v>1098.0</v>
       </c>
       <c r="B63">
-        <v>2.9452945701566902e-30</v>
+        <v>3.4672188375457224e-5</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64">
-        <v>187488.0</v>
+        <v>1116.0</v>
       </c>
       <c r="B64">
-        <v>3.182564729991209e-30</v>
+        <v>3.636248561900159e-5</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65">
-        <v>190512.0</v>
+        <v>1134.0</v>
       </c>
       <c r="B65">
-        <v>3.427010276562514e-30</v>
+        <v>3.8073774472397115e-5</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66">
-        <v>193536.0</v>
+        <v>1152.0</v>
       </c>
       <c r="B66">
-        <v>3.6786312098706045e-30</v>
+        <v>3.980363038272179e-5</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67">
-        <v>196560.0</v>
+        <v>1170.0</v>
       </c>
       <c r="B67">
-        <v>3.937427529915482e-30</v>
+        <v>4.154897124596074e-5</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68">
-        <v>199584.0</v>
+        <v>1188.0</v>
       </c>
       <c r="B68">
-        <v>4.203399236697148e-30</v>
+        <v>4.330671495809912e-5</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69">
-        <v>202608.0</v>
+        <v>1206.0</v>
       </c>
       <c r="B69">
-        <v>4.476546330215597e-30</v>
+        <v>4.507377941512205e-5</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70">
-        <v>205632.0</v>
+        <v>1224.0</v>
       </c>
       <c r="B70">
-        <v>4.756868810470834e-30</v>
+        <v>4.684708251301468e-5</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71">
-        <v>208656.0</v>
+        <v>1242.0</v>
       </c>
       <c r="B71">
-        <v>5.044366677462855e-30</v>
+        <v>4.862354214776213e-5</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72">
-        <v>211680.0</v>
+        <v>1260.0</v>
       </c>
       <c r="B72">
-        <v>5.3390399311916645e-30</v>
+        <v>5.040341327929911e-5</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73">
-        <v>214704.0</v>
+        <v>1278.0</v>
       </c>
       <c r="B73">
-        <v>5.640888571657261e-30</v>
+        <v>5.2191483940737014e-5</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74">
-        <v>217728.0</v>
+        <v>1296.0</v>
       </c>
       <c r="B74">
-        <v>5.949912598859641e-30</v>
+        <v>5.398544997616967e-5</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75">
-        <v>220752.0</v>
+        <v>1314.0</v>
       </c>
       <c r="B75">
-        <v>6.26611201279881e-30</v>
+        <v>5.578271443240817e-5</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76">
-        <v>223776.0</v>
+        <v>1332.0</v>
       </c>
       <c r="B76">
-        <v>6.589486813474762e-30</v>
+        <v>5.758068035626356e-5</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77">
-        <v>226800.0</v>
+        <v>1350.0</v>
       </c>
       <c r="B77">
-        <v>6.920037000887505e-30</v>
+        <v>5.937675079454694e-5</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78">
-        <v>229824.0</v>
+        <v>1368.0</v>
       </c>
       <c r="B78">
-        <v>7.257762575037029e-30</v>
+        <v>6.116832879406937e-5</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79">
-        <v>232848.0</v>
+        <v>1386.0</v>
       </c>
       <c r="B79">
-        <v>7.602663535923346e-30</v>
+        <v>6.295281740164191e-5</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80">
-        <v>235872.0</v>
+        <v>1404.0</v>
       </c>
       <c r="B80">
-        <v>7.954739883546444e-30</v>
+        <v>6.473243779977704e-5</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81">
-        <v>238896.0</v>
+        <v>1422.0</v>
       </c>
       <c r="B81">
-        <v>8.31399161790633e-30</v>
+        <v>6.651141602490723e-5</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82">
-        <v>241920.0</v>
+        <v>1440.0</v>
       </c>
       <c r="B82">
-        <v>8.680418739002999e-30</v>
+        <v>6.828769610239772e-5</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83">
-        <v>244944.0</v>
+        <v>1458.0</v>
       </c>
       <c r="B83">
-        <v>9.054021246836457e-30</v>
+        <v>7.005918692133484e-5</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84">
-        <v>247968.0</v>
+        <v>1476.0</v>
       </c>
       <c r="B84">
-        <v>9.434799141406703e-30</v>
+        <v>7.182379737080502e-5</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85">
-        <v>250992.0</v>
+        <v>1494.0</v>
       </c>
       <c r="B85">
-        <v>9.822752422713734e-30</v>
+        <v>7.35794363398946e-5</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86">
-        <v>254016.0</v>
+        <v>1512.0</v>
       </c>
       <c r="B86">
-        <v>1.0217881090757549e-29</v>
+        <v>7.532401271768999e-5</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87">
-        <v>257040.0</v>
+        <v>1530.0</v>
       </c>
       <c r="B87">
-        <v>1.0620185145538153e-29</v>
+        <v>7.705543539327754e-5</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>260064.0</v>
+        <v>1548.0</v>
       </c>
       <c r="B88">
-        <v>1.1029664587055543e-29</v>
+        <v>7.877161325574363e-5</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
-        <v>263088.0</v>
+        <v>1566.0</v>
       </c>
       <c r="B89">
-        <v>1.1446319415309722e-29</v>
+        <v>8.04753468802255e-5</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90">
-        <v>266112.0</v>
+        <v>1584.0</v>
       </c>
       <c r="B90">
-        <v>1.1870149630300683e-29</v>
+        <v>8.21709740213913e-5</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91">
-        <v>269136.0</v>
+        <v>1602.0</v>
       </c>
       <c r="B91">
-        <v>1.230115523202843e-29</v>
+        <v>8.385719149176108e-5</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92">
-        <v>272160.0</v>
+        <v>1620.0</v>
       </c>
       <c r="B92">
-        <v>1.2739336220492965e-29</v>
+        <v>8.55326828021886e-5</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93">
-        <v>275184.0</v>
+        <v>1638.0</v>
       </c>
       <c r="B93">
-        <v>1.3184692595694287e-29</v>
+        <v>8.719613146352768e-5</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94">
-        <v>278208.0</v>
+        <v>1656.0</v>
       </c>
       <c r="B94">
-        <v>1.3637224357632392e-29</v>
+        <v>8.884622098663212e-5</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95">
-        <v>281232.0</v>
+        <v>1674.0</v>
       </c>
       <c r="B95">
-        <v>1.4096931506307285e-29</v>
+        <v>9.04816348823557e-5</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96">
-        <v>284256.0</v>
+        <v>1692.0</v>
       </c>
       <c r="B96">
-        <v>1.4563814041718967e-29</v>
+        <v>9.21010566615522e-5</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97">
-        <v>287280.0</v>
+        <v>1710.0</v>
       </c>
       <c r="B97">
-        <v>1.503787196386743e-29</v>
+        <v>9.370316983507544e-5</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98">
-        <v>290304.0</v>
+        <v>1728.0</v>
       </c>
       <c r="B98">
-        <v>1.551910527275269e-29</v>
+        <v>9.528665791377921e-5</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99">
-        <v>293328.0</v>
+        <v>1746.0</v>
       </c>
       <c r="B99">
-        <v>1.6007513968374724e-29</v>
+        <v>9.685142014742942e-5</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100">
-        <v>296352.0</v>
+        <v>1764.0</v>
       </c>
       <c r="B100">
-        <v>1.6503098050733553e-29</v>
+        <v>9.840252893161273e-5</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101">
-        <v>299376.0</v>
+        <v>1782.0</v>
       </c>
       <c r="B101">
-        <v>1.7005857519829156e-29</v>
+        <v>9.994014742069898e-5</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102">
-        <v>302400.0</v>
+        <v>1800.0</v>
       </c>
       <c r="B102">
-        <v>1.7515792375661556e-29</v>
+        <v>0.0001014636121431105</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103">
-        <v>305424.0</v>
+        <v>1818.0</v>
       </c>
       <c r="B103">
-        <v>1.803290261823074e-29</v>
+        <v>0.00010297225962726954</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104">
-        <v>308448.0</v>
+        <v>1836.0</v>
       </c>
       <c r="B104">
-        <v>1.8557188247536712e-29</v>
+        <v>0.00010446542640159842</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105">
-        <v>311472.0</v>
+        <v>1854.0</v>
       </c>
       <c r="B105">
-        <v>1.908864926357947e-29</v>
+        <v>0.00010594244899451943</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106">
-        <v>314496.0</v>
+        <v>1872.0</v>
       </c>
       <c r="B106">
-        <v>1.962728566635901e-29</v>
+        <v>0.00010740266393445484</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107">
-        <v>317520.0</v>
+        <v>1890.0</v>
       </c>
       <c r="B107">
-        <v>2.0173097455875345e-29</v>
+        <v>0.00010884540774982696</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108">
-        <v>320544.0</v>
+        <v>1908.0</v>
       </c>
       <c r="B108">
-        <v>2.0726084632128456e-29</v>
+        <v>0.00011027001696905805</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109">
-        <v>323568.0</v>
+        <v>1926.0</v>
       </c>
       <c r="B109">
-        <v>2.1286247195118356e-29</v>
+        <v>0.00011167589360552763</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110">
-        <v>326592.0</v>
+        <v>1944.0</v>
       </c>
       <c r="B110">
-        <v>2.185358514484505e-29</v>
+        <v>0.00011306657979367595</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111">
-        <v>329616.0</v>
+        <v>1962.0</v>
       </c>
       <c r="B111">
-        <v>2.2428098481308523e-29</v>
+        <v>0.00011444405422730516</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112">
-        <v>332640.0</v>
+        <v>1980.0</v>
       </c>
       <c r="B112">
-        <v>2.300978720450878e-29</v>
+        <v>0.00011580782983931163</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113">
-        <v>335664.0</v>
+        <v>1998.0</v>
       </c>
       <c r="B113">
-        <v>2.3598651314445828e-29</v>
+        <v>0.00011715741956259185</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114">
-        <v>338688.0</v>
+        <v>2016.0</v>
       </c>
       <c r="B114">
-        <v>2.419469081111966e-29</v>
+        <v>0.00011849233633004222</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115">
-        <v>341712.0</v>
+        <v>2034.0</v>
       </c>
       <c r="B115">
-        <v>2.479790569453028e-29</v>
+        <v>0.00011981209307455914</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116">
-        <v>344736.0</v>
+        <v>2052.0</v>
       </c>
       <c r="B116">
-        <v>2.5408295964677684e-29</v>
+        <v>0.00012111620272903909</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117">
-        <v>347760.0</v>
+        <v>2070.0</v>
       </c>
       <c r="B117">
-        <v>2.6025861621561874e-29</v>
+        <v>0.00012240417822637846</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118">
-        <v>350784.0</v>
+        <v>2088.0</v>
       </c>
       <c r="B118">
-        <v>2.6650602665182856e-29</v>
+        <v>0.0001236755324994737</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119">
-        <v>353808.0</v>
+        <v>2106.0</v>
       </c>
       <c r="B119">
-        <v>2.728251909554062e-29</v>
+        <v>0.00012492977848122124</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120">
-        <v>356832.0</v>
+        <v>2124.0</v>
       </c>
       <c r="B120">
-        <v>2.7921610912635164e-29</v>
+        <v>0.00012616642910451747</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121">
-        <v>359856.0</v>
+        <v>2142.0</v>
       </c>
       <c r="B121">
-        <v>2.85678781164665e-29</v>
+        <v>0.00012738499730225887</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122">
-        <v>362880.0</v>
+        <v>2160.0</v>
       </c>
       <c r="B122">
-        <v>2.922132070703463e-29</v>
+        <v>0.0001285856404483997</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123">
-        <v>365904.0</v>
+        <v>2178.0</v>
       </c>
       <c r="B123">
-        <v>2.9881938684339535e-29</v>
+        <v>0.00012977361370717952</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124">
-        <v>368928.0</v>
+        <v>2196.0</v>
       </c>
       <c r="B124">
-        <v>3.054973204838123e-29</v>
+        <v>0.00013094981378402148</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125">
-        <v>371952.0</v>
+        <v>2214.0</v>
       </c>
       <c r="B125">
-        <v>3.1224700799159723e-29</v>
+        <v>0.00013211378686526742</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126">
-        <v>374976.0</v>
+        <v>2232.0</v>
       </c>
       <c r="B126">
-        <v>3.190684493667499e-29</v>
+        <v>0.00013326507913725903</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127">
-        <v>378000.0</v>
+        <v>2250.0</v>
       </c>
       <c r="B127">
-        <v>3.2596164460927047e-29</v>
+        <v>0.0001344032367863381</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128">
-        <v>381024.0</v>
+        <v>2268.0</v>
       </c>
       <c r="B128">
-        <v>3.3292659371915886e-29</v>
+        <v>0.00013552780599884636</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129">
-        <v>384048.0</v>
+        <v>2286.0</v>
       </c>
       <c r="B129">
-        <v>3.3996329669641507e-29</v>
+        <v>0.0001366383329611256</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130">
-        <v>387072.0</v>
+        <v>2304.0</v>
       </c>
       <c r="B130">
-        <v>3.470717535410393e-29</v>
+        <v>0.00013773436385951755</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131">
-        <v>390096.0</v>
+        <v>2322.0</v>
       </c>
       <c r="B131">
-        <v>3.5425196425303137e-29</v>
+        <v>0.00013881544488036397</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132">
-        <v>393120.0</v>
+        <v>2340.0</v>
       </c>
       <c r="B132">
-        <v>3.615039288323912e-29</v>
+        <v>0.00013988112221000664</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133">
-        <v>396144.0</v>
+        <v>2358.0</v>
       </c>
       <c r="B133">
-        <v>3.6882764727911886e-29</v>
+        <v>0.00014093094203478727</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134">
-        <v>399168.0</v>
+        <v>2376.0</v>
       </c>
       <c r="B134">
-        <v>3.762231195932144e-29</v>
+        <v>0.00014196445054104768</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135">
-        <v>402192.0</v>
+        <v>2394.0</v>
       </c>
       <c r="B135">
-        <v>3.8369034577467783e-29</v>
+        <v>0.00014298274799702082</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136">
-        <v>405216.0</v>
+        <v>2412.0</v>
       </c>
       <c r="B136">
-        <v>3.912293258235091e-29</v>
+        <v>0.00014399032524575685</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137">
-        <v>408240.0</v>
+        <v>2430.0</v>
       </c>
       <c r="B137">
-        <v>3.9884005973970833e-29</v>
+        <v>0.000144987236381216</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138">
-        <v>411264.0</v>
+        <v>2448.0</v>
       </c>
       <c r="B138">
-        <v>4.0652254752327547e-29</v>
+        <v>0.00014597318502194257</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139">
-        <v>414288.0</v>
+        <v>2466.0</v>
       </c>
       <c r="B139">
-        <v>4.142767891742103e-29</v>
+        <v>0.00014694787478648102</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140">
-        <v>417312.0</v>
+        <v>2484.0</v>
       </c>
       <c r="B140">
-        <v>4.2210278469251296e-29</v>
+        <v>0.00014791100929337564</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141">
-        <v>420336.0</v>
+        <v>2502.0</v>
       </c>
       <c r="B141">
-        <v>4.300005340781837e-29</v>
+        <v>0.00014886229216117084</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142">
-        <v>423360.0</v>
+        <v>2520.0</v>
       </c>
       <c r="B142">
-        <v>4.3797003733122214e-29</v>
+        <v>0.00014980142700841097</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143">
-        <v>426384.0</v>
+        <v>2538.0</v>
       </c>
       <c r="B143">
-        <v>4.4601129445162857e-29</v>
+        <v>0.0001507281174536404</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144">
-        <v>429408.0</v>
+        <v>2556.0</v>
       </c>
       <c r="B144">
-        <v>4.541243054394027e-29</v>
+        <v>0.00015164206711540352</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145">
-        <v>432432.0</v>
+        <v>2574.0</v>
       </c>
       <c r="B145">
-        <v>4.6230907029454485e-29</v>
+        <v>0.00015254297961224468</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146">
-        <v>435456.0</v>
+        <v>2592.0</v>
       </c>
       <c r="B146">
-        <v>4.705655890170549e-29</v>
+        <v>0.00015343055856270824</v>
       </c>
     </row>
     <row r="147" spans="1:2">
       <c r="A147">
-        <v>438480.0</v>
+        <v>2610.0</v>
       </c>
       <c r="B147">
-        <v>4.7889386160693256e-29</v>
+        <v>0.00015430450758533858</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148">
-        <v>441504.0</v>
+        <v>2628.0</v>
       </c>
       <c r="B148">
-        <v>4.8729388806417827e-29</v>
+        <v>0.0001551666741781442</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149">
-        <v>444528.0</v>
+        <v>2646.0</v>
       </c>
       <c r="B149">
-        <v>4.957656683887918e-29</v>
+        <v>0.00015601948371143093</v>
       </c>
     </row>
     <row r="150" spans="1:2">
       <c r="A150">
-        <v>447552.0</v>
+        <v>2664.0</v>
       </c>
       <c r="B150">
-        <v>5.043092025807733e-29</v>
+        <v>0.0001568627749303893</v>
       </c>
     </row>
     <row r="151" spans="1:2">
       <c r="A151">
-        <v>450576.0</v>
+        <v>2682.0</v>
       </c>
       <c r="B151">
-        <v>5.129244906401224e-29</v>
+        <v>0.00015769637964390394</v>
       </c>
     </row>
     <row r="152" spans="1:2">
       <c r="A152">
-        <v>453600.0</v>
+        <v>2700.0</v>
       </c>
       <c r="B152">
-        <v>5.216115325668396e-29</v>
+        <v>0.00015852012966085946</v>
       </c>
     </row>
     <row r="153" spans="1:2">
       <c r="A153">
-        <v>456624.0</v>
+        <v>2718.0</v>
       </c>
       <c r="B153">
-        <v>5.303703283609246e-29</v>
+        <v>0.00015933385679014065</v>
       </c>
     </row>
     <row r="154" spans="1:2">
       <c r="A154">
-        <v>459648.0</v>
+        <v>2736.0</v>
       </c>
       <c r="B154">
-        <v>5.392008780223772e-29</v>
+        <v>0.000160137392840632</v>
       </c>
     </row>
     <row r="155" spans="1:2">
       <c r="A155">
-        <v>462672.0</v>
+        <v>2754.0</v>
       </c>
       <c r="B155">
-        <v>5.481031815511979e-29</v>
+        <v>0.00016093056962121821</v>
       </c>
     </row>
     <row r="156" spans="1:2">
       <c r="A156">
-        <v>465696.0</v>
+        <v>2772.0</v>
       </c>
       <c r="B156">
-        <v>5.570772389473866e-29</v>
+        <v>0.00016171321894078397</v>
       </c>
     </row>
     <row r="157" spans="1:2">
       <c r="A157">
-        <v>468720.0</v>
+        <v>2790.0</v>
       </c>
       <c r="B157">
-        <v>5.661809846852962e-29</v>
+        <v>0.00016248517260821388</v>
       </c>
     </row>
     <row r="158" spans="1:2">
       <c r="A158">
-        <v>471744.0</v>
+        <v>2808.0</v>
       </c>
       <c r="B158">
-        <v>5.770781064765378e-29</v>
+        <v>0.00016324626243239263</v>
       </c>
     </row>
     <row r="159" spans="1:2">
       <c r="A159">
-        <v>474768.0</v>
+        <v>2826.0</v>
       </c>
       <c r="B159">
-        <v>5.88103815603307e-29</v>
+        <v>0.00016399632022220484</v>
       </c>
     </row>
     <row r="160" spans="1:2">
       <c r="A160">
-        <v>477792.0</v>
+        <v>2844.0</v>
       </c>
       <c r="B160">
-        <v>5.992587776474248e-29</v>
+        <v>0.0001647352531262744</v>
       </c>
     </row>
     <row r="161" spans="1:2">
       <c r="A161">
-        <v>480816.0</v>
+        <v>2862.0</v>
       </c>
       <c r="B161">
-        <v>6.10543658190712e-29</v>
+        <v>0.0001654650944538941</v>
       </c>
     </row>
     <row r="162" spans="1:2">
       <c r="A162">
-        <v>483840.0</v>
+        <v>2880.0</v>
       </c>
       <c r="B162">
-        <v>6.219591228149893e-29</v>
+        <v>0.0001661867441721289</v>
       </c>
     </row>
     <row r="163" spans="1:2">
       <c r="A163">
-        <v>486864.0</v>
+        <v>2898.0</v>
       </c>
       <c r="B163">
-        <v>6.335058371020771e-29</v>
+        <v>0.0001669001016950484</v>
       </c>
     </row>
     <row r="164" spans="1:2">
       <c r="A164">
-        <v>489888.0</v>
+        <v>2916.0</v>
       </c>
       <c r="B164">
-        <v>6.451844666337968e-29</v>
+        <v>0.00016760506643672234</v>
       </c>
     </row>
     <row r="165" spans="1:2">
       <c r="A165">
-        <v>492912.0</v>
+        <v>2934.0</v>
       </c>
       <c r="B165">
-        <v>6.569956769919686e-29</v>
+        <v>0.0001683015378112204</v>
       </c>
     </row>
     <row r="166" spans="1:2">
       <c r="A166">
-        <v>495936.0</v>
+        <v>2952.0</v>
       </c>
       <c r="B166">
-        <v>6.689401337584136e-29</v>
+        <v>0.0001689894152326123</v>
       </c>
     </row>
     <row r="167" spans="1:2">
       <c r="A167">
-        <v>498960.0</v>
+        <v>2970.0</v>
       </c>
       <c r="B167">
-        <v>6.810185025149525e-29</v>
+        <v>0.00016966859811496756</v>
       </c>
     </row>
     <row r="168" spans="1:2">
       <c r="A168">
-        <v>501984.0</v>
+        <v>2988.0</v>
       </c>
       <c r="B168">
-        <v>6.932314488434058e-29</v>
+        <v>0.00017033898587235605</v>
       </c>
     </row>
     <row r="169" spans="1:2">
       <c r="A169">
-        <v>505008.0</v>
+        <v>3006.0</v>
       </c>
       <c r="B169">
-        <v>7.055796383255948e-29</v>
+        <v>0.00017100047791884733</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170">
-        <v>508032.0</v>
+        <v>3024.0</v>
       </c>
       <c r="B170">
-        <v>7.180637365433399e-29</v>
+        <v>0.00017165297366851114</v>
       </c>
     </row>
     <row r="171" spans="1:2">
       <c r="A171">
-        <v>511056.0</v>
+        <v>3042.0</v>
       </c>
       <c r="B171">
-        <v>7.306844090784617e-29</v>
+        <v>0.0001722963725354171</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172">
-        <v>514080.0</v>
+        <v>3060.0</v>
       </c>
       <c r="B172">
-        <v>7.434423215127812e-29</v>
+        <v>0.00017293057393363492</v>
       </c>
     </row>
     <row r="173" spans="1:2">
       <c r="A173">
-        <v>517104.0</v>
+        <v>3078.0</v>
       </c>
       <c r="B173">
-        <v>7.563381394281195e-29</v>
+        <v>0.0001735556169221694</v>
       </c>
     </row>
     <row r="174" spans="1:2">
       <c r="A174">
-        <v>520128.0</v>
+        <v>3096.0</v>
       </c>
       <c r="B174">
-        <v>7.693725284062965e-29</v>
+        <v>0.00017417237491783986</v>
       </c>
     </row>
     <row r="175" spans="1:2">
       <c r="A175">
-        <v>523152.0</v>
+        <v>3114.0</v>
       </c>
       <c r="B175">
-        <v>7.825461540291339e-29</v>
+        <v>0.00017478111082145715</v>
       </c>
     </row>
     <row r="176" spans="1:2">
       <c r="A176">
-        <v>526176.0</v>
+        <v>3132.0</v>
       </c>
       <c r="B176">
-        <v>7.958596818784519e-29</v>
+        <v>0.00017538193770036092</v>
       </c>
     </row>
     <row r="177" spans="1:2">
       <c r="A177">
-        <v>529200.0</v>
+        <v>3150.0</v>
       </c>
       <c r="B177">
-        <v>8.093137775360713e-29</v>
+        <v>0.0001759749686218906</v>
       </c>
     </row>
     <row r="178" spans="1:2">
       <c r="A178">
-        <v>532224.0</v>
+        <v>3168.0</v>
       </c>
       <c r="B178">
-        <v>8.22909106583813e-29</v>
+        <v>0.00017656031665338564</v>
       </c>
     </row>
     <row r="179" spans="1:2">
       <c r="A179">
-        <v>535248.0</v>
+        <v>3186.0</v>
       </c>
       <c r="B179">
-        <v>8.366463346034976e-29</v>
+        <v>0.00017713809486218568</v>
       </c>
     </row>
     <row r="180" spans="1:2">
       <c r="A180">
-        <v>538272.0</v>
+        <v>3204.0</v>
       </c>
       <c r="B180">
-        <v>8.505261271769462e-29</v>
+        <v>0.00017770841631563014</v>
       </c>
     </row>
     <row r="181" spans="1:2">
       <c r="A181">
-        <v>541296.0</v>
+        <v>3222.0</v>
       </c>
       <c r="B181">
-        <v>8.645491498859793e-29</v>
+        <v>0.00017827139408105853</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182">
-        <v>544320.0</v>
+        <v>3240.0</v>
       </c>
       <c r="B182">
-        <v>8.787160683124173e-29</v>
+        <v>0.00017882714122581037</v>
       </c>
     </row>
     <row r="183" spans="1:2">
       <c r="A183">
-        <v>547344.0</v>
+        <v>3258.0</v>
       </c>
       <c r="B183">
-        <v>8.930275480380819e-29</v>
+        <v>0.00017937577081722516</v>
       </c>
     </row>
     <row r="184" spans="1:2">
       <c r="A184">
-        <v>550368.0</v>
+        <v>3276.0</v>
       </c>
       <c r="B184">
-        <v>9.074842546447928e-29</v>
+        <v>0.00017991739592264241</v>
       </c>
     </row>
     <row r="185" spans="1:2">
       <c r="A185">
-        <v>553392.0</v>
+        <v>3294.0</v>
       </c>
       <c r="B185">
-        <v>9.220868537143718e-29</v>
+        <v>0.00018045212960940163</v>
       </c>
     </row>
     <row r="186" spans="1:2">
       <c r="A186">
-        <v>556416.0</v>
+        <v>3312.0</v>
       </c>
       <c r="B186">
-        <v>9.368360108286388e-29</v>
+        <v>0.0001809800849448423</v>
       </c>
     </row>
     <row r="187" spans="1:2">
       <c r="A187">
-        <v>559440.0</v>
+        <v>3330.0</v>
       </c>
       <c r="B187">
-        <v>9.517323915694153e-29</v>
+        <v>0.00018150137499630396</v>
       </c>
     </row>
     <row r="188" spans="1:2">
       <c r="A188">
-        <v>562464.0</v>
+        <v>3348.0</v>
       </c>
       <c r="B188">
-        <v>9.667766615185213e-29</v>
+        <v>0.0001820161128311261</v>
       </c>
     </row>
     <row r="189" spans="1:2">
       <c r="A189">
-        <v>565488.0</v>
+        <v>3366.0</v>
       </c>
       <c r="B189">
-        <v>9.819694862577782e-29</v>
+        <v>0.00018252441151664822</v>
       </c>
     </row>
     <row r="190" spans="1:2">
       <c r="A190">
-        <v>568512.0</v>
+        <v>3384.0</v>
       </c>
       <c r="B190">
-        <v>9.973115313690062e-29</v>
+        <v>0.00018302638412020982</v>
       </c>
     </row>
     <row r="191" spans="1:2">
       <c r="A191">
-        <v>571536.0</v>
+        <v>3402.0</v>
       </c>
       <c r="B191">
-        <v>1.0128034624340264e-28</v>
+        <v>0.00018352214370915044</v>
       </c>
     </row>
     <row r="192" spans="1:2">
       <c r="A192">
-        <v>574560.0</v>
+        <v>3420.0</v>
       </c>
       <c r="B192">
-        <v>1.02844594503466e-28</v>
+        <v>0.00018401180335080958</v>
       </c>
     </row>
     <row r="193" spans="1:2">
       <c r="A193">
-        <v>577584.0</v>
+        <v>3438.0</v>
       </c>
       <c r="B193">
-        <v>1.0442396447527265e-28</v>
+        <v>0.0001844954761125267</v>
       </c>
     </row>
     <row r="194" spans="1:2">
       <c r="A194">
-        <v>580608.0</v>
+        <v>3456.0</v>
       </c>
       <c r="B194">
-        <v>1.060185227170048e-28</v>
+        <v>0.00018497327506164133</v>
       </c>
     </row>
     <row r="195" spans="1:2">
       <c r="A195">
-        <v>583632.0</v>
+        <v>3474.0</v>
       </c>
       <c r="B195">
-        <v>1.0762833578684443e-28</v>
+        <v>0.00018544481903778266</v>
       </c>
     </row>
     <row r="196" spans="1:2">
       <c r="A196">
-        <v>586656.0</v>
+        <v>3492.0</v>
       </c>
       <c r="B196">
-        <v>1.0925347024297372e-28</v>
+        <v>0.00018590965526222978</v>
       </c>
     </row>
     <row r="197" spans="1:2">
       <c r="A197">
-        <v>589680.0</v>
+        <v>3510.0</v>
       </c>
       <c r="B197">
-        <v>1.1089399264357464e-28</v>
+        <v>0.000186368090921813</v>
       </c>
     </row>
     <row r="198" spans="1:2">
       <c r="A198">
-        <v>592704.0</v>
+        <v>3528.0</v>
       </c>
       <c r="B198">
-        <v>1.125499695468293e-28</v>
+        <v>0.0001868204379437719</v>
       </c>
     </row>
     <row r="199" spans="1:2">
       <c r="A199">
-        <v>595728.0</v>
+        <v>3546.0</v>
       </c>
       <c r="B199">
-        <v>1.142214675109198e-28</v>
+        <v>0.00018726700825534608</v>
       </c>
     </row>
     <row r="200" spans="1:2">
       <c r="A200">
-        <v>598752.0</v>
+        <v>3564.0</v>
       </c>
       <c r="B200">
-        <v>1.1590855309402821e-28</v>
+        <v>0.0001877081137837751</v>
       </c>
     </row>
     <row r="201" spans="1:2">
       <c r="A201">
-        <v>601776.0</v>
+        <v>3582.0</v>
       </c>
       <c r="B201">
-        <v>1.1761129285433658e-28</v>
+        <v>0.00018814406645629856</v>
       </c>
     </row>
     <row r="202" spans="1:2">
       <c r="A202">
-        <v>604800.0</v>
+        <v>3600.0</v>
       </c>
       <c r="B202">
-        <v>1.1932975335002704e-28</v>
+        <v>0.00018857517820015604</v>
       </c>
     </row>
   </sheetData>

</xml_diff>